<commit_message>
ContrPro GC: update Application for Payment, Bid Estimator, Project Operations
Content additions to the three core GC deliverables (each grew ~7KB over
the v1.0 launch versions).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/contrpro/files/packages/complete/gc/GC_Application_for_Payment.xlsx
+++ b/contrpro/files/packages/complete/gc/GC_Application_for_Payment.xlsx
@@ -31,6 +31,42 @@
     <definedName name="G703Total_Retainage">'G-703 Pay App'!$L$65</definedName>
     <definedName name="G703Total_Previous">'G-703 Pay App'!$E$65</definedName>
     <definedName name="G703Total_NetDue">'G-703 Pay App'!$N$65</definedName>
+    <definedName name="CSI_Divisions">'CSI Reference'!$A$5:$A$39</definedName>
+    <definedName name="CSI_Div_00">'CSI Reference'!$D$5:$D$12</definedName>
+    <definedName name="CSI_Div_01">'CSI Reference'!$D$13:$D$21</definedName>
+    <definedName name="CSI_Div_02">'CSI Reference'!$D$22:$D$28</definedName>
+    <definedName name="CSI_Div_03">'CSI Reference'!$D$29:$D$36</definedName>
+    <definedName name="CSI_Div_04">'CSI Reference'!$D$37:$D$43</definedName>
+    <definedName name="CSI_Div_05">'CSI Reference'!$D$44:$D$49</definedName>
+    <definedName name="CSI_Div_06">'CSI Reference'!$D$50:$D$56</definedName>
+    <definedName name="CSI_Div_07">'CSI Reference'!$D$57:$D$65</definedName>
+    <definedName name="CSI_Div_08">'CSI Reference'!$D$66:$D$73</definedName>
+    <definedName name="CSI_Div_09">'CSI Reference'!$D$74:$D$80</definedName>
+    <definedName name="CSI_Div_10">'CSI Reference'!$D$81:$D$88</definedName>
+    <definedName name="CSI_Div_11">'CSI Reference'!$D$89:$D$96</definedName>
+    <definedName name="CSI_Div_12">'CSI Reference'!$D$97:$D$103</definedName>
+    <definedName name="CSI_Div_13">'CSI Reference'!$D$104:$D$108</definedName>
+    <definedName name="CSI_Div_14">'CSI Reference'!$D$109:$D$115</definedName>
+    <definedName name="CSI_Div_21">'CSI Reference'!$D$116:$D$119</definedName>
+    <definedName name="CSI_Div_22">'CSI Reference'!$D$120:$D$125</definedName>
+    <definedName name="CSI_Div_23">'CSI Reference'!$D$126:$D$133</definedName>
+    <definedName name="CSI_Div_25">'CSI Reference'!$D$134:$D$136</definedName>
+    <definedName name="CSI_Div_26">'CSI Reference'!$D$137:$D$141</definedName>
+    <definedName name="CSI_Div_27">'CSI Reference'!$D$142:$D$146</definedName>
+    <definedName name="CSI_Div_28">'CSI Reference'!$D$147:$D$151</definedName>
+    <definedName name="CSI_Div_31">'CSI Reference'!$D$152:$D$158</definedName>
+    <definedName name="CSI_Div_32">'CSI Reference'!$D$159:$D$163</definedName>
+    <definedName name="CSI_Div_33">'CSI Reference'!$D$164:$D$171</definedName>
+    <definedName name="CSI_Div_34">'CSI Reference'!$D$172:$D$176</definedName>
+    <definedName name="CSI_Div_35">'CSI Reference'!$D$177:$D$182</definedName>
+    <definedName name="CSI_Div_40">'CSI Reference'!$D$183:$D$186</definedName>
+    <definedName name="CSI_Div_41">'CSI Reference'!$D$187:$D$191</definedName>
+    <definedName name="CSI_Div_42">'CSI Reference'!$D$192:$D$194</definedName>
+    <definedName name="CSI_Div_43">'CSI Reference'!$D$195:$D$198</definedName>
+    <definedName name="CSI_Div_44">'CSI Reference'!$D$199:$D$202</definedName>
+    <definedName name="CSI_Div_45">'CSI Reference'!$D$203:$D$203</definedName>
+    <definedName name="CSI_Div_46">'CSI Reference'!$D$204:$D$210</definedName>
+    <definedName name="CSI_Div_48">'CSI Reference'!$D$211:$D$212</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +79,7 @@
     <numFmt numFmtId="165" formatCode="_($* #,##0.00_);_($* (#,##0.00);_($* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,6 +126,19 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001E3A5F"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -135,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -186,6 +235,13 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1051,7 +1107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1065,6 +1121,8 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1135,6 +1193,16 @@
       <c r="K4" s="15" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="L4" s="31" t="inlineStr">
+        <is>
+          <t>CSI Div</t>
+        </is>
+      </c>
+      <c r="M4" s="31" t="inlineStr">
+        <is>
+          <t>CSI Subdivision</t>
         </is>
       </c>
     </row>
@@ -2851,12 +2919,18 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="C5:C64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"01,02,03,04,05,06,07,08,09,10,11,12,13,14,21,22,23,25,26,27,28,31,32,33"</formula1>
     </dataValidation>
     <dataValidation sqref="J5:J64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Base Contract,Change Order,Allowance,Bond,Insurance,Tax,General Conditions,Self-Perform,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L5:L60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid CSI Division" error="Pick a division from the dropdown (sourced from the CSI Reference tab)." promptTitle="CSI MasterFormat Division" prompt="Pick the CSI Level 1 division for this line item." type="list">
+      <formula1>=CSI_Divisions</formula1>
+    </dataValidation>
+    <dataValidation sqref="M5:M60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid CSI Subdivision" error="Pick a subdivision that belongs to the division in the CSI Div column. Re-pick the division first if you don't see your subdivision." promptTitle="CSI MasterFormat Subdivision" prompt="Filtered by the division code in the CSI Div column (this same row)." type="list">
+      <formula1>=INDIRECT("CSI_Div_" &amp; $L5)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2869,7 +2943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:P65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2886,6 +2960,8 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2985,6 +3061,16 @@
       <c r="N4" s="15" t="inlineStr">
         <is>
           <t>This Period Net Due ($)</t>
+        </is>
+      </c>
+      <c r="O4" s="31" t="inlineStr">
+        <is>
+          <t>CSI Div</t>
+        </is>
+      </c>
+      <c r="P4" s="31" t="inlineStr">
+        <is>
+          <t>CSI Subdivision</t>
         </is>
       </c>
     </row>
@@ -6346,6 +6432,14 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="O5:O60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid CSI Division" error="Pick a division from the dropdown (sourced from the CSI Reference tab)." promptTitle="CSI MasterFormat Division" prompt="Pick the CSI Level 1 division for this line item." type="list">
+      <formula1>=CSI_Divisions</formula1>
+    </dataValidation>
+    <dataValidation sqref="P5:P60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid CSI Subdivision" error="Pick a subdivision that belongs to the division in the CSI Div column. Re-pick the division first if you don't see your subdivision." promptTitle="CSI MasterFormat Subdivision" prompt="Filtered by the division code in the CSI Div column (this same row)." type="list">
+      <formula1>=INDIRECT("CSI_Div_" &amp; $O5)</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9724,309 +9818,3943 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:E212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>CSI MasterFormat Divisions</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A1" s="32" t="inlineStr">
+        <is>
+          <t>CSI MasterFormat 2020 — Divisions and Subdivisions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="33" t="inlineStr">
+        <is>
+          <t>Reference data for the bid + log workbooks. Do not delete columns A, B, D, or E — the dropdowns in the other tabs source from these named ranges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Div Code</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>Division Title</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>Subdiv Code</t>
+        </is>
+      </c>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>Subdivision Title (parent division shown in col C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Procurement and Contracting Requirements</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>00 10 00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Solicitation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B3" s="24" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>General Requirements</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>00 20 00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Instructions for Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Existing Conditions</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>00 30 00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Available Information</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Concrete</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>00 40 00</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Procurement Forms and Supplements</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Masonry</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>00 50 00</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Contracting Forms and Supplements</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Metals</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>00 60 00</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Project Forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>06</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Wood, Plastics, and Composites</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>00 70 00</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Conditions of the Contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>07</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Thermal and Moisture Protection</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>00 80 00</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Revisions, Clarifications, and Modifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>08</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Openings</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>01 10 00</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>09</t>
         </is>
       </c>
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Finishes</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>01 20 00</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Price and Payment Procedures</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Specialties</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>01 30 00</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Administrative Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Equipment</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>01 40 00</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Quality Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Furnishings</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>01 50 00</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Temporary Facilities and Controls</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Special Construction</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>01 60 00</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Product Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Conveying Equipment</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="24" t="inlineStr">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>01 70 00</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Execution and Closeout Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="B17" s="24" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Fire Suppression</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>01 80 00</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Performance Requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="B18" s="24" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Plumbing</t>
         </is>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>01 90 00</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Life Cycle Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="B19" s="24" t="inlineStr">
-        <is>
-          <t>HVAC</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Heating, Ventilating, and Air Conditioning (HVAC)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>02 20 00</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="B20" s="24" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Integrated Automation</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="24" t="inlineStr">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>02 30 00</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Subsurface Investigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="B21" s="24" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Electrical</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>02 40 00</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Demolition and Structure Moving</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Communications</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>02 50 00</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Site Remediation</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B23" s="24" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Electronic Safety and Security</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="24" t="inlineStr">
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>02 60 00</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Contaminated Site Material Removal</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
-      <c r="B24" s="24" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Earthwork</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>02 70 00</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Water Remediation</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="B25" s="24" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>Exterior Improvements</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="24" t="inlineStr">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>02 80 00</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Facility Remediation</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="B26" s="24" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Utilities</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>03 10 00</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Concrete Forming and Accessories</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>03 20 00</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Concrete Reinforcing</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Waterway and Marine Construction</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>03 30 00</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Cast-in-Place Concrete</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Process Interconnections</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>03 40 00</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Precast Concrete</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Material Processing and Handling Equipment</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>03 50 00</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Cast Decks and Underlayment</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Process Heating, Cooling, and Drying Equipment</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>03 60 00</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Grouting</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Process Gas and Liquid Handling, Purification, and Storage Equipment</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>03 70 00</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Mass Concrete</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Pollution and Waste Control Equipment</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>03 80 00</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Concrete Cutting and Boring</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Industry-Specific Manufacturing Equipment</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>04 01 00</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Maintenance of Masonry</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Water and Wastewater Equipment</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>04 05 00</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Common Work Results for Masonry</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Electrical Power Generation</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>04 20 00</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Unit Masonry</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>04 40 00</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Stone Assemblies</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>04 50 00</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Refractory Masonry</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>04 60 00</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Corrosion-Resistant Masonry</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>04 70 00</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Manufactured Masonry</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>05 10 00</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Structural Metal Framing</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>05 20 00</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Metal Joists</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>05 30 00</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Metal Decking</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>05 40 00</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Cold-Formed Metal Framing</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>05 50 00</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Metal Fabrications</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>05 70 00</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Decorative Metal</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>06 10 00</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Rough Carpentry</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>06 20 00</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Finish Carpentry</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>06 40 00</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Architectural Woodwork</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>06 50 00</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Structural Plastics</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>06 60 00</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Plastic Fabrications</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>06 70 00</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Structural Composites</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>06 80 00</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Composite Fabrications</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>07 10 00</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Dampproofing and Waterproofing</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>07 20 00</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Thermal Protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>07 30 00</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Steep Slope Roofing</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>07 40 00</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Roofing and Siding Panels</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>07 50 00</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Membrane Roofing</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>07 60 00</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Flashing and Sheet Metal</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>07 70 00</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Roof and Wall Specialties and Accessories</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>07 80 00</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Fire and Smoke Protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>07 90 00</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Joint Protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>08 10 00</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Doors and Frames</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>08 30 00</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Specialty Doors and Frames</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>08 40 00</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Entrances, Storefronts, and Curtain Walls</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>08 50 00</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>08 60 00</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Roof Windows and Skylights</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>08 70 00</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>08 80 00</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Glazing</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>08 90 00</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Louvers and Vents</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>09 20 00</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Plaster and Gypsum Board</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>09 30 00</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Tiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>09 50 00</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Ceilings</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>09 60 00</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Flooring</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>09 70 00</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Wall Finishes</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>09 80 00</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Acoustic Treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>09 90 00</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Painting and Coating</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>10 10 00</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Information Specialties</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>10 20 00</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Interior Specialties</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>10 30 00</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Fireplaces and Stoves</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>10 40 00</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Safety Specialties</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>10 50 00</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Storage Specialties</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>10 60 00</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Pedestrian Specialties</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>10 70 00</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Exterior Specialties</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>10 80 00</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Other Specialties</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>11 10 00</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Vehicle and Pedestrian Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>11 20 00</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Commercial Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>11 30 00</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Residential Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>11 40 00</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Foodservice Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>11 50 00</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Educational and Scientific Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>11 60 00</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Entertainment Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>11 70 00</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Healthcare Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>11 80 00</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Collection and Disposal Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>12 10 00</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>12 20 00</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Window Treatments</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>12 30 00</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Casework</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>12 40 00</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Furnishings and Accessories</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>12 50 00</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>12 60 00</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Multiple Seating</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>12 90 00</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Other Furnishings</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>13 10 00</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Special Facility Components</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>13 20 00</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Special Purpose Rooms</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>13 30 00</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Special Structures</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>13 40 00</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Integrated Construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>13 50 00</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Special Instrumentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>14 10 00</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Dumbwaiters</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>14 20 00</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Elevators</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>14 30 00</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Escalators and Moving Walks</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>14 40 00</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Lifts</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>14 70 00</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Turntables</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>14 80 00</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Scaffolding</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>14 90 00</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Other Conveying Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>21 10 00</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Water-Based Fire-Suppression Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>21 20 00</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Fire-Extinguishing Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>21 30 00</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Fire Pumps</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>21 40 00</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Fire-Suppression Water Storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>22 10 00</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Plumbing Piping and Pumps</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>22 30 00</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Plumbing Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>22 40 00</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Plumbing Fixtures</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>22 50 00</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Pool and Fountain Plumbing Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>22 60 00</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Gas and Vacuum Systems for Laboratory and Healthcare Facilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>22 70 00</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Off-Grade Water Storage and Distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>23 10 00</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Facility Fuel Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>23 20 00</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>HVAC Piping and Pumps</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>23 30 00</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>HVAC Air Distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>23 40 00</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>HVAC Air Cleaning Devices</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>23 50 00</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Central Heating Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>23 60 00</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Central Cooling Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>23 70 00</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Central HVAC Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>23 80 00</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Decentralized HVAC Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>25 10 00</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Integrated Automation Network Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>25 30 00</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Integrated Automation Instrumentation and Terminal Devices</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>25 50 00</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Integrated Automation Facility Controls</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>26 10 00</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Medium-Voltage Electrical Distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>26 20 00</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Low-Voltage Electrical Distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>26 30 00</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Facility Electrical Power Generating and Storing Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>26 40 00</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Electrical and Cathodic Protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>26 50 00</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>27 10 00</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Structured Cabling</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>27 20 00</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Data Communications</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>27 30 00</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Voice Communications</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>27 40 00</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Audio-Video Communications</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>27 50 00</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Distributed Communications and Monitoring Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>28 10 00</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Access Control</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>28 20 00</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Video Surveillance</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>28 30 00</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Security Detection, Alarm, and Monitoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>28 40 00</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Electronic Detection and Alarm</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>28 50 00</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Specialized Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>31 10 00</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Site Clearing</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>31 20 00</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Earth Moving</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>31 30 00</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Earthwork Methods</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>31 40 00</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Shoring and Underpinning</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>31 50 00</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Excavation Support and Protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>31 60 00</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Special Foundations and Load-Bearing Elements</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>31 70 00</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Tunneling and Mining</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>32 10 00</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Bases, Ballasts, and Paving</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>32 30 00</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Site Improvements</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>32 70 00</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Wetlands</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>32 80 00</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Irrigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>32 90 00</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Planting</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>33 10 00</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Water Utilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>33 20 00</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Wells</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>33 30 00</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Sanitary Sewerage Utilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>33 40 00</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Storm Drainage Utilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>33 50 00</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Fuel Distribution Utilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>33 60 00</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Hydronic and Steam Energy Utilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>33 70 00</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Electrical Utilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>33 80 00</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Communications Utilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>34 10 00</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Guideways/Railways</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>34 20 00</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Traction Power</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>34 40 00</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Transportation Signaling and Control Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>34 70 00</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Transportation Construction and Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>34 80 00</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Bridges</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>35 10 00</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Waterway and Marine Signaling and Control Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>35 20 00</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Waterway and Marine Construction and Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>35 30 00</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Coastal Construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>35 40 00</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Waterway Construction and Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>35 50 00</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Marine Construction and Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>35 70 00</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Dam Construction and Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>40 10 00</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Gas and Vapor Process Piping</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>40 20 00</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Liquids Process Piping</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>40 30 00</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Solid and Mixed Materials Piping and Chutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>40 40 00</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Process Piping and Equipment Protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>41 10 00</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Bulk Material Processing Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>41 20 00</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Piece Material Handling Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>41 30 00</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Manufacturing Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>41 40 00</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Container Processing and Packaging</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>41 50 00</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Material Storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>42 10 00</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Process Heating Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>42 20 00</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Process Cooling Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>42 30 00</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Process Drying Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>43 10 00</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Gas Handling Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>43 20 00</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Liquid Handling Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>43 30 00</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Gas and Liquid Purification Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>43 40 00</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Gas and Liquid Storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>44 10 00</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Air Pollution Control</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>44 20 00</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Noise Pollution Control</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>44 40 00</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Water Treatment Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>44 50 00</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Solid Waste Control</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>45 10 00</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Specific-Use Manufacturing Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>46 20 00</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Water and Wastewater Preliminary Treatment Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>46 30 00</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Water and Wastewater Chemical Feed Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>46 40 00</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Water and Wastewater Clarification and Mixing Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>46 50 00</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Water and Wastewater Secondary Treatment Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>46 60 00</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Water and Wastewater Advanced Treatment Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>46 70 00</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Water and Wastewater Residuals Handling and Treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>46 80 00</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Water and Wastewater Disinfection</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>48 10 00</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Electrical Power Generation Equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>48 70 00</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Electrical Power Generation Testing</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>